<commit_message>
Update seller promo page
</commit_message>
<xml_diff>
--- a/quote-bsd.xlsx
+++ b/quote-bsd.xlsx
@@ -1208,15 +1208,27 @@
           <t>카드</t>
         </is>
       </c>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="8" t="n"/>
-      <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="n"/>
+      <c r="C23" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>카드 할인 TBD · 확정 시 업데이트 (할인율 최대 15%, 셀러 분담 최대 50%)</t>
+          <t>지마켓꾹현대·지마켓삼성·KB국민·NH농협·롯데·비씨·IBK나라사랑 · G마켓/옥션 동일 · 디지털 등 일부 카테고리 별도 스킴 · 예산 소진 시 조기 종료 가능</t>
         </is>
       </c>
       <c r="J23" s="4" t="n"/>

</xml_diff>